<commit_message>
Add reconciliation business rule tests
</commit_message>
<xml_diff>
--- a/data/processed/client_report.xlsx
+++ b/data/processed/client_report.xlsx
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -561,10 +561,15 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>has_payment</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>difference</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>reconciliation_status</t>
         </is>
@@ -593,10 +598,13 @@
       <c r="F2" t="n">
         <v>250</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
@@ -625,10 +633,13 @@
       <c r="F3" t="n">
         <v>100</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
         <v>25.5</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>PARTIAL_PAYMENT</t>
         </is>
@@ -657,10 +668,13 @@
       <c r="F4" t="n">
         <v>300</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
         <v>0</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
@@ -689,10 +703,13 @@
       <c r="F5" t="n">
         <v>450</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
@@ -721,10 +738,13 @@
       <c r="F6" t="n">
         <v>175.75</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
         <v>0</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
@@ -753,10 +773,13 @@
       <c r="F7" t="n">
         <v>90</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
         <v>0</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
@@ -785,10 +808,13 @@
       <c r="F8" t="n">
         <v>520</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
         <v>0</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
@@ -817,10 +843,13 @@
       <c r="F9" t="n">
         <v>210</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
         <v>0</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>CANCELLED_WITH_PAYMENT</t>
         </is>
@@ -849,10 +878,13 @@
       <c r="F10" t="n">
         <v>50</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="n">
         <v>35.5</v>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>PARTIAL_PAYMENT</t>
         </is>
@@ -881,10 +913,13 @@
       <c r="F11" t="n">
         <v>640</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
         <v>0</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
@@ -901,7 +936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -937,10 +972,15 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>has_payment</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>difference</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>reconciliation_status</t>
         </is>
@@ -969,10 +1009,13 @@
       <c r="F2" t="n">
         <v>100</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
         <v>25.5</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>PARTIAL_PAYMENT</t>
         </is>
@@ -1001,10 +1044,13 @@
       <c r="F3" t="n">
         <v>210</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>CANCELLED_WITH_PAYMENT</t>
         </is>
@@ -1033,10 +1079,13 @@
       <c r="F4" t="n">
         <v>50</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
         <v>35.5</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>PARTIAL_PAYMENT</t>
         </is>

</xml_diff>